<commit_message>
Excel: completar pruebas de combos con Espada corta como arma principal
Añade las 7 combinaciones de Espada corta (sola, dual con Daga/Espada
corta/Maza pequeña, +Escudo pequeño/normal/grande), igual que se hizo
antes con Daga. Tabla queda con 14 filas en total.
</commit_message>
<xml_diff>
--- a/pruebas_combos_slime.xlsx
+++ b/pruebas_combos_slime.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1415,15 +1415,774 @@
         <v>63</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta + —</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>614.1</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.885</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="n"/>
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>4/4/4/2/0</t>
+        </is>
+      </c>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>10/11/11/6/0</t>
+        </is>
+      </c>
+      <c r="P9" s="6" t="inlineStr">
+        <is>
+          <t>17/18/15/7/0</t>
+        </is>
+      </c>
+      <c r="Q9" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="S9" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="T9" s="6" t="inlineStr">
+        <is>
+          <t>5.37–6.64 → 6.00–7.21</t>
+        </is>
+      </c>
+      <c r="U9" s="6" t="inlineStr"/>
+      <c r="V9" s="6" t="inlineStr">
+        <is>
+          <t>1.81–2.37</t>
+        </is>
+      </c>
+      <c r="W9" s="6" t="inlineStr">
+        <is>
+          <t>2.59–3.42</t>
+        </is>
+      </c>
+      <c r="X9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>Material de Slime (Normal)×1, Material de Slime (Defectuoso)×1</t>
+        </is>
+      </c>
+      <c r="AC9" s="3" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="AD9" s="3" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AE9" s="6" t="n">
+        <v>52</v>
+      </c>
+    </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>* Mano 2 idéntica a Mano 1: el log de Daga+Daga(dual) no distingue qué mano golpeó en cada línea (mismo arma en ambas manos).</t>
-        </is>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta + Daga (dual)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>810.5</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>0.767</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Daga</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>0.176</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>1.542</v>
+      </c>
+      <c r="N10" s="6" t="inlineStr">
+        <is>
+          <t>6/7/7/4/0</t>
+        </is>
+      </c>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>10/9/10/8/0</t>
+        </is>
+      </c>
+      <c r="P10" s="6" t="inlineStr">
+        <is>
+          <t>16/15/15/12/0</t>
+        </is>
+      </c>
+      <c r="Q10" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="R10" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="S10" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="T10" s="6" t="inlineStr">
+        <is>
+          <t>5.36–6.72 → 5.84–7.16</t>
+        </is>
+      </c>
+      <c r="U10" s="6" t="inlineStr">
+        <is>
+          <t>4.24–5.04 → 4.49–5.35</t>
+        </is>
+      </c>
+      <c r="V10" s="6" t="inlineStr">
+        <is>
+          <t>1.75–2.19</t>
+        </is>
+      </c>
+      <c r="W10" s="6" t="inlineStr">
+        <is>
+          <t>2.74–3.32</t>
+        </is>
+      </c>
+      <c r="X10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB10" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AC10" s="3" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="AD10" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="AE10" s="6" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta + Espada corta (dual)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>768.1</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0.868</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta*</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>0.868</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="M11" s="3" t="n">
+        <v>1.417</v>
+      </c>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>4/3/4/0/0</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>8/7/8/4/0</t>
+        </is>
+      </c>
+      <c r="P11" s="6" t="inlineStr">
+        <is>
+          <t>13/12/11/8/0</t>
+        </is>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="T11" s="6" t="inlineStr">
+        <is>
+          <t>5.35–6.76 → 5.66–7.02</t>
+        </is>
+      </c>
+      <c r="U11" s="6" t="inlineStr"/>
+      <c r="V11" s="6" t="inlineStr">
+        <is>
+          <t>1.58–1.86</t>
+        </is>
+      </c>
+      <c r="W11" s="6" t="inlineStr">
+        <is>
+          <t>2.56–3.25</t>
+        </is>
+      </c>
+      <c r="X11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z11" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB11" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AC11" s="3" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="AD11" s="3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="AE11" s="6" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta + Maza pequeña (dual)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>6.81</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>750.9</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>5.77</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>0.929</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M12" s="3" t="n">
+        <v>1.367</v>
+      </c>
+      <c r="N12" s="6" t="inlineStr">
+        <is>
+          <t>5/5/7/1/0</t>
+        </is>
+      </c>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>10/10/10/2/0</t>
+        </is>
+      </c>
+      <c r="P12" s="6" t="inlineStr">
+        <is>
+          <t>14/13/12/3/0</t>
+        </is>
+      </c>
+      <c r="Q12" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="R12" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="S12" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="T12" s="6" t="inlineStr">
+        <is>
+          <t>5.54–6.49 → 5.80–7.03</t>
+        </is>
+      </c>
+      <c r="U12" s="6" t="inlineStr">
+        <is>
+          <t>5.30–6.22 → 5.31–6.51</t>
+        </is>
+      </c>
+      <c r="V12" s="6" t="inlineStr">
+        <is>
+          <t>1.56–1.98</t>
+        </is>
+      </c>
+      <c r="W12" s="6" t="inlineStr">
+        <is>
+          <t>2.60–3.28</t>
+        </is>
+      </c>
+      <c r="X12" s="5" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="Y12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z12" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA12" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB12" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AC12" s="3" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="AD12" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AE12" s="6" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta + Escudo pequeño</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>610.6</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="3" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="M13" s="3" t="n">
+        <v>1.045</v>
+      </c>
+      <c r="N13" s="6" t="inlineStr">
+        <is>
+          <t>4/6/4/0/0</t>
+        </is>
+      </c>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>11/16/10/2/0</t>
+        </is>
+      </c>
+      <c r="P13" s="6" t="inlineStr">
+        <is>
+          <t>15/22/13/5/0</t>
+        </is>
+      </c>
+      <c r="Q13" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="S13" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="T13" s="6" t="inlineStr">
+        <is>
+          <t>5.39–6.53 → 5.70–6.50</t>
+        </is>
+      </c>
+      <c r="U13" s="6" t="inlineStr"/>
+      <c r="V13" s="6" t="inlineStr">
+        <is>
+          <t>1.15–1.49</t>
+        </is>
+      </c>
+      <c r="W13" s="6" t="inlineStr">
+        <is>
+          <t>2.56–3.46</t>
+        </is>
+      </c>
+      <c r="X13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AC13" s="3" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="AD13" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AE13" s="6" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta + Escudo normal</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>563.2</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>5.82</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="3" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>0.968</v>
+      </c>
+      <c r="N14" s="6" t="inlineStr">
+        <is>
+          <t>4/7/6/1/0</t>
+        </is>
+      </c>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>8/13/8/1/0</t>
+        </is>
+      </c>
+      <c r="P14" s="6" t="inlineStr">
+        <is>
+          <t>14/22/13/3/0</t>
+        </is>
+      </c>
+      <c r="Q14" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="R14" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="S14" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="T14" s="6" t="inlineStr">
+        <is>
+          <t>5.45–6.77 → 5.79–7.07</t>
+        </is>
+      </c>
+      <c r="U14" s="6" t="inlineStr"/>
+      <c r="V14" s="6" t="inlineStr">
+        <is>
+          <t>0.90–1.13</t>
+        </is>
+      </c>
+      <c r="W14" s="6" t="inlineStr">
+        <is>
+          <t>2.59–3.43</t>
+        </is>
+      </c>
+      <c r="X14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z14" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>Material de Slime (Defectuoso)×1</t>
+        </is>
+      </c>
+      <c r="AC14" s="3" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="AD14" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="AE14" s="6" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta + Escudo grande</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>505</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0.865</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M15" s="3" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="N15" s="6" t="inlineStr">
+        <is>
+          <t>4/7/4/1/0</t>
+        </is>
+      </c>
+      <c r="O15" s="6" t="inlineStr">
+        <is>
+          <t>10/16/10/2/0</t>
+        </is>
+      </c>
+      <c r="P15" s="6" t="inlineStr">
+        <is>
+          <t>15/27/14/4/0</t>
+        </is>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="T15" s="6" t="inlineStr">
+        <is>
+          <t>5.36–6.72 → 5.74–7.03</t>
+        </is>
+      </c>
+      <c r="U15" s="6" t="inlineStr"/>
+      <c r="V15" s="6" t="inlineStr">
+        <is>
+          <t>0.65–0.84</t>
+        </is>
+      </c>
+      <c r="W15" s="6" t="inlineStr">
+        <is>
+          <t>2.56–3.38</t>
+        </is>
+      </c>
+      <c r="X15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB15" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AC15" s="3" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="AD15" s="3" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="AE15" s="6" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>* Mano 2 idéntica a Mano 1: el log de Daga+Daga(dual) no distingue qué mano golpeó en cada línea (mismo arma en ambas manos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>% Aturdir proc solo cuenta golpes de la mano capaz de aturdir (aturdir base &gt; 0); las demás manos siempre dan 0%.</t>
         </is>

</xml_diff>

<commit_message>
Excel: completar pruebas de combos con Espada larga como arma principal
Añade las 4 combinaciones de Espada larga (sola, +Escudo pequeño/normal/
grande; no admite dual-wield). Tabla queda con 18 filas: Daga (7),
Espada corta (7) y Espada larga (4) completas.
</commit_message>
<xml_diff>
--- a/pruebas_combos_slime.xlsx
+++ b/pruebas_combos_slime.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE18"/>
+  <dimension ref="A1:AE22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2174,15 +2174,427 @@
         <v>52</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Espada larga + —</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>658</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Espada larga</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="n"/>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" s="6" t="inlineStr">
+        <is>
+          <t>3/3/4/0/0</t>
+        </is>
+      </c>
+      <c r="O16" s="6" t="inlineStr">
+        <is>
+          <t>10/11/8/2/0</t>
+        </is>
+      </c>
+      <c r="P16" s="6" t="inlineStr">
+        <is>
+          <t>16/17/11/3/0</t>
+        </is>
+      </c>
+      <c r="Q16" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="R16" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="S16" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="T16" s="6" t="inlineStr">
+        <is>
+          <t>6.37–7.49 → 6.99–8.44</t>
+        </is>
+      </c>
+      <c r="U16" s="6" t="inlineStr"/>
+      <c r="V16" s="6" t="inlineStr">
+        <is>
+          <t>1.86–2.38</t>
+        </is>
+      </c>
+      <c r="W16" s="6" t="inlineStr">
+        <is>
+          <t>2.57–3.46</t>
+        </is>
+      </c>
+      <c r="X16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB16" s="2" t="inlineStr">
+        <is>
+          <t>Material de Slime (Defectuoso)×1 (+1 cristal roto/perdido, no contabilizado)</t>
+        </is>
+      </c>
+      <c r="AC16" s="3" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="AD16" s="3" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="AE16" s="6" t="n">
+        <v>45</v>
+      </c>
+    </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>* Mano 2 idéntica a Mano 1: el log de Daga+Daga(dual) no distingue qué mano golpeó en cada línea (mismo arma en ambas manos).</t>
-        </is>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Espada larga + Escudo pequeño</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>684.7</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Espada larga</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0.927</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="3" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="M17" s="3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>5/9/7/2/0</t>
+        </is>
+      </c>
+      <c r="O17" s="6" t="inlineStr">
+        <is>
+          <t>10/17/8/3/0</t>
+        </is>
+      </c>
+      <c r="P17" s="6" t="inlineStr">
+        <is>
+          <t>15/24/13/7/0</t>
+        </is>
+      </c>
+      <c r="Q17" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="R17" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="S17" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="T17" s="6" t="inlineStr">
+        <is>
+          <t>6.24–7.78 → 6.99–8.33</t>
+        </is>
+      </c>
+      <c r="U17" s="6" t="inlineStr"/>
+      <c r="V17" s="6" t="inlineStr">
+        <is>
+          <t>1.21–1.46</t>
+        </is>
+      </c>
+      <c r="W17" s="6" t="inlineStr">
+        <is>
+          <t>2.52–3.40</t>
+        </is>
+      </c>
+      <c r="X17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z17" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA17" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB17" s="2" t="inlineStr">
+        <is>
+          <t>ninguno (+1 cristal roto/perdido, no contabilizado)</t>
+        </is>
+      </c>
+      <c r="AC17" s="3" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="AD17" s="3" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="AE17" s="6" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Espada larga + Escudo normal</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>626.6</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Espada larga</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>0.952</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="6" t="n"/>
+      <c r="J18" s="6" t="n"/>
+      <c r="K18" s="6" t="n"/>
+      <c r="L18" s="3" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="M18" s="3" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="N18" s="6" t="inlineStr">
+        <is>
+          <t>6/10/7/1/0</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="inlineStr">
+        <is>
+          <t>11/19/13/2/0</t>
+        </is>
+      </c>
+      <c r="P18" s="6" t="inlineStr">
+        <is>
+          <t>15/25/15/4/0</t>
+        </is>
+      </c>
+      <c r="Q18" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="R18" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="S18" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="T18" s="6" t="inlineStr">
+        <is>
+          <t>6.29–7.93 → 6.73–8.11</t>
+        </is>
+      </c>
+      <c r="U18" s="6" t="inlineStr"/>
+      <c r="V18" s="6" t="inlineStr">
+        <is>
+          <t>0.97–1.21</t>
+        </is>
+      </c>
+      <c r="W18" s="6" t="inlineStr">
+        <is>
+          <t>2.58–3.46</t>
+        </is>
+      </c>
+      <c r="X18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA18" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB18" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AC18" s="3" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="AD18" s="3" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="AE18" s="6" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Espada larga + Escudo grande</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>578.4</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Espada larga</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M19" s="3" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>4/7/6/3/0</t>
+        </is>
+      </c>
+      <c r="O19" s="6" t="inlineStr">
+        <is>
+          <t>10/15/10/6/0</t>
+        </is>
+      </c>
+      <c r="P19" s="6" t="inlineStr">
+        <is>
+          <t>16/24/15/6/0</t>
+        </is>
+      </c>
+      <c r="Q19" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="R19" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="S19" s="6" t="n">
+        <v>61</v>
+      </c>
+      <c r="T19" s="6" t="inlineStr">
+        <is>
+          <t>6.44–7.79 → 6.98–8.35</t>
+        </is>
+      </c>
+      <c r="U19" s="6" t="inlineStr"/>
+      <c r="V19" s="6" t="inlineStr">
+        <is>
+          <t>0.69–0.85</t>
+        </is>
+      </c>
+      <c r="W19" s="6" t="inlineStr">
+        <is>
+          <t>2.58–3.33</t>
+        </is>
+      </c>
+      <c r="X19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z19" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB19" s="2" t="inlineStr">
+        <is>
+          <t>Material de Slime (Defectuoso)×1</t>
+        </is>
+      </c>
+      <c r="AC19" s="3" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="AD19" s="3" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="AE19" s="6" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>* Mano 2 idéntica a Mano 1: el log de Daga+Daga(dual) no distingue qué mano golpeó en cada línea (mismo arma en ambas manos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>% Aturdir proc solo cuenta golpes de la mano capaz de aturdir (aturdir base &gt; 0); las demás manos siempre dan 0%.</t>
         </is>

</xml_diff>

<commit_message>
Fix retraso ATB no perceptible con barra baja + Excel pruebas Maza pequeña
El retraso parcial por aturdir recortaba la barra ATB a 0 con maxf(),
así que si el enemigo ya estaba con la barra baja el golpe aturdidor no
tenía ningún efecto perceptible (quedaba igual que sin aturdir). Ahora
resta el mismo tiempo sin recorte, dejándola ir a negativo si hace
falta, igual que ya hacía el aturdimiento completo por crítico.

Incluye el Excel con las 7 combinaciones de Maza pequeña como arma
principal (sola, dual con Daga/Espada corta/Maza pequeña,
+Escudo pequeño/normal/grande) y la columna nueva "Aturdir proc (n/n)".
</commit_message>
<xml_diff>
--- a/pruebas_combos_slime.xlsx
+++ b/pruebas_combos_slime.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE22"/>
+  <dimension ref="A1:AF29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -490,13 +490,14 @@
     <col width="18" customWidth="1" min="22" max="22"/>
     <col width="18" customWidth="1" min="23" max="23"/>
     <col width="10" customWidth="1" min="24" max="24"/>
-    <col width="8" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
     <col width="8" customWidth="1" min="26" max="26"/>
     <col width="8" customWidth="1" min="27" max="27"/>
-    <col width="26" customWidth="1" min="28" max="28"/>
-    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="8" customWidth="1" min="28" max="28"/>
+    <col width="26" customWidth="1" min="29" max="29"/>
     <col width="12" customWidth="1" min="30" max="30"/>
-    <col width="10" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="31" max="31"/>
+    <col width="10" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -622,35 +623,40 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
+          <t>Aturdir proc (n/n)</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>Cristales Cat1</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Cristales Cat2</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Cristales Cat3</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Drops obtenidos</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Dmg medio recibido/golpe</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Poder medio slimes</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>n (golpes muestreados)</t>
         </is>
@@ -735,27 +741,32 @@
       <c r="X2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y2" s="6" t="n">
+      <c r="Y2" s="6" t="inlineStr">
+        <is>
+          <t>0/64</t>
+        </is>
+      </c>
+      <c r="Z2" s="6" t="n">
         <v>4</v>
-      </c>
-      <c r="Z2" s="6" t="n">
-        <v>2</v>
       </c>
       <c r="AA2" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AB2" s="2" t="inlineStr">
+      <c r="AB2" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC2" s="2" t="inlineStr">
         <is>
           <t>ninguno</t>
         </is>
       </c>
-      <c r="AC2" s="3" t="n">
+      <c r="AD2" s="3" t="n">
         <v>2.33</v>
       </c>
-      <c r="AD2" s="3" t="n">
+      <c r="AE2" s="3" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="AE2" s="6" t="n">
+      <c r="AF2" s="6" t="n">
         <v>64</v>
       </c>
     </row>
@@ -848,27 +859,32 @@
       <c r="X3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y3" s="6" t="n">
+      <c r="Y3" s="6" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="Z3" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="Z3" s="6" t="n">
+      <c r="AA3" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="AA3" s="6" t="n">
+      <c r="AB3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="AB3" s="2" t="inlineStr">
+      <c r="AC3" s="2" t="inlineStr">
         <is>
           <t>ninguno</t>
         </is>
       </c>
-      <c r="AC3" s="3" t="n">
+      <c r="AD3" s="3" t="n">
         <v>2.35</v>
       </c>
-      <c r="AD3" s="3" t="n">
+      <c r="AE3" s="3" t="n">
         <v>0.99</v>
       </c>
-      <c r="AE3" s="6" t="n">
+      <c r="AF3" s="6" t="n">
         <v>62</v>
       </c>
     </row>
@@ -965,27 +981,32 @@
       <c r="X4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y4" s="6" t="n">
+      <c r="Y4" s="6" t="inlineStr">
+        <is>
+          <t>0/61</t>
+        </is>
+      </c>
+      <c r="Z4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Z4" s="6" t="n">
+      <c r="AA4" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="AA4" s="6" t="n">
+      <c r="AB4" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AB4" s="2" t="inlineStr">
+      <c r="AC4" s="2" t="inlineStr">
         <is>
           <t>Material de Slime (Defectuoso)×1</t>
         </is>
       </c>
-      <c r="AC4" s="3" t="n">
+      <c r="AD4" s="3" t="n">
         <v>2.24</v>
       </c>
-      <c r="AD4" s="3" t="n">
+      <c r="AE4" s="3" t="n">
         <v>0.98</v>
       </c>
-      <c r="AE4" s="6" t="n">
+      <c r="AF4" s="6" t="n">
         <v>61</v>
       </c>
     </row>
@@ -1082,27 +1103,32 @@
       <c r="X5" s="5" t="n">
         <v>0.07099999999999999</v>
       </c>
-      <c r="Y5" s="6" t="n">
-        <v>2</v>
+      <c r="Y5" s="6" t="inlineStr">
+        <is>
+          <t>2/28</t>
+        </is>
       </c>
       <c r="Z5" s="6" t="n">
         <v>2</v>
       </c>
       <c r="AA5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB5" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="AB5" s="2" t="inlineStr">
+      <c r="AC5" s="2" t="inlineStr">
         <is>
           <t>Material de Slime (Defectuoso)×1</t>
         </is>
       </c>
-      <c r="AC5" s="3" t="n">
+      <c r="AD5" s="3" t="n">
         <v>2.61</v>
       </c>
-      <c r="AD5" s="3" t="n">
+      <c r="AE5" s="3" t="n">
         <v>1.03</v>
       </c>
-      <c r="AE5" s="6" t="n">
+      <c r="AF5" s="6" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1185,27 +1211,32 @@
       <c r="X6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y6" s="6" t="n">
+      <c r="Y6" s="6" t="inlineStr">
+        <is>
+          <t>0/71</t>
+        </is>
+      </c>
+      <c r="Z6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="Z6" s="6" t="n">
+      <c r="AA6" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="AA6" s="6" t="n">
+      <c r="AB6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AB6" s="2" t="inlineStr">
+      <c r="AC6" s="2" t="inlineStr">
         <is>
           <t>ninguno</t>
         </is>
       </c>
-      <c r="AC6" s="3" t="n">
+      <c r="AD6" s="3" t="n">
         <v>2.66</v>
       </c>
-      <c r="AD6" s="3" t="n">
+      <c r="AE6" s="3" t="n">
         <v>1.04</v>
       </c>
-      <c r="AE6" s="6" t="n">
+      <c r="AF6" s="6" t="n">
         <v>71</v>
       </c>
     </row>
@@ -1288,27 +1319,32 @@
       <c r="X7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y7" s="6" t="n">
+      <c r="Y7" s="6" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="Z7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Z7" s="6" t="n">
+      <c r="AA7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AA7" s="6" t="n">
+      <c r="AB7" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="AB7" s="2" t="inlineStr">
+      <c r="AC7" s="2" t="inlineStr">
         <is>
           <t>ninguno</t>
         </is>
       </c>
-      <c r="AC7" s="3" t="n">
+      <c r="AD7" s="3" t="n">
         <v>2.62</v>
       </c>
-      <c r="AD7" s="3" t="n">
+      <c r="AE7" s="3" t="n">
         <v>1.05</v>
       </c>
-      <c r="AE7" s="6" t="n">
+      <c r="AF7" s="6" t="n">
         <v>62</v>
       </c>
     </row>
@@ -1391,27 +1427,32 @@
       <c r="X8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y8" s="6" t="n">
+      <c r="Y8" s="6" t="inlineStr">
+        <is>
+          <t>0/63</t>
+        </is>
+      </c>
+      <c r="Z8" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Z8" s="6" t="n">
+      <c r="AA8" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="AA8" s="6" t="n">
+      <c r="AB8" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AB8" s="2" t="inlineStr">
+      <c r="AC8" s="2" t="inlineStr">
         <is>
           <t>ninguno</t>
         </is>
       </c>
-      <c r="AC8" s="3" t="n">
+      <c r="AD8" s="3" t="n">
         <v>2.6</v>
       </c>
-      <c r="AD8" s="3" t="n">
+      <c r="AE8" s="3" t="n">
         <v>1.02</v>
       </c>
-      <c r="AE8" s="6" t="n">
+      <c r="AF8" s="6" t="n">
         <v>63</v>
       </c>
     </row>
@@ -1494,27 +1535,32 @@
       <c r="X9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y9" s="6" t="n">
+      <c r="Y9" s="6" t="inlineStr">
+        <is>
+          <t>0/52</t>
+        </is>
+      </c>
+      <c r="Z9" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="Z9" s="6" t="n">
+      <c r="AA9" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AA9" s="6" t="n">
+      <c r="AB9" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="AB9" s="2" t="inlineStr">
+      <c r="AC9" s="2" t="inlineStr">
         <is>
           <t>Material de Slime (Normal)×1, Material de Slime (Defectuoso)×1</t>
         </is>
       </c>
-      <c r="AC9" s="3" t="n">
+      <c r="AD9" s="3" t="n">
         <v>2.9</v>
       </c>
-      <c r="AD9" s="3" t="n">
+      <c r="AE9" s="3" t="n">
         <v>0.97</v>
       </c>
-      <c r="AE9" s="6" t="n">
+      <c r="AF9" s="6" t="n">
         <v>52</v>
       </c>
     </row>
@@ -1611,27 +1657,32 @@
       <c r="X10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y10" s="6" t="n">
+      <c r="Y10" s="6" t="inlineStr">
+        <is>
+          <t>0/55</t>
+        </is>
+      </c>
+      <c r="Z10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Z10" s="6" t="n">
+      <c r="AA10" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="AA10" s="6" t="n">
+      <c r="AB10" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="AB10" s="2" t="inlineStr">
+      <c r="AC10" s="2" t="inlineStr">
         <is>
           <t>ninguno</t>
         </is>
       </c>
-      <c r="AC10" s="3" t="n">
+      <c r="AD10" s="3" t="n">
         <v>2.69</v>
       </c>
-      <c r="AD10" s="3" t="n">
+      <c r="AE10" s="3" t="n">
         <v>1.02</v>
       </c>
-      <c r="AE10" s="6" t="n">
+      <c r="AF10" s="6" t="n">
         <v>55</v>
       </c>
     </row>
@@ -1724,27 +1775,32 @@
       <c r="X11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y11" s="6" t="n">
+      <c r="Y11" s="6" t="inlineStr">
+        <is>
+          <t>0/53</t>
+        </is>
+      </c>
+      <c r="Z11" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="Z11" s="6" t="n">
+      <c r="AA11" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="AA11" s="6" t="n">
+      <c r="AB11" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="AB11" s="2" t="inlineStr">
+      <c r="AC11" s="2" t="inlineStr">
         <is>
           <t>ninguno</t>
         </is>
       </c>
-      <c r="AC11" s="3" t="n">
+      <c r="AD11" s="3" t="n">
         <v>2.42</v>
       </c>
-      <c r="AD11" s="3" t="n">
+      <c r="AE11" s="3" t="n">
         <v>0.85</v>
       </c>
-      <c r="AE11" s="6" t="n">
+      <c r="AF11" s="6" t="n">
         <v>53</v>
       </c>
     </row>
@@ -1841,27 +1897,32 @@
       <c r="X12" s="5" t="n">
         <v>0.125</v>
       </c>
-      <c r="Y12" s="6" t="n">
+      <c r="Y12" s="6" t="inlineStr">
+        <is>
+          <t>3/24</t>
+        </is>
+      </c>
+      <c r="Z12" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Z12" s="6" t="n">
+      <c r="AA12" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="AA12" s="6" t="n">
+      <c r="AB12" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="AB12" s="2" t="inlineStr">
+      <c r="AC12" s="2" t="inlineStr">
         <is>
           <t>ninguno</t>
         </is>
       </c>
-      <c r="AC12" s="3" t="n">
+      <c r="AD12" s="3" t="n">
         <v>2.81</v>
       </c>
-      <c r="AD12" s="3" t="n">
+      <c r="AE12" s="3" t="n">
         <v>0.99</v>
       </c>
-      <c r="AE12" s="6" t="n">
+      <c r="AF12" s="6" t="n">
         <v>52</v>
       </c>
     </row>
@@ -1944,27 +2005,32 @@
       <c r="X13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y13" s="6" t="n">
+      <c r="Y13" s="6" t="inlineStr">
+        <is>
+          <t>0/51</t>
+        </is>
+      </c>
+      <c r="Z13" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="Z13" s="6" t="n">
+      <c r="AA13" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AA13" s="6" t="n">
+      <c r="AB13" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="AB13" s="2" t="inlineStr">
+      <c r="AC13" s="2" t="inlineStr">
         <is>
           <t>ninguno</t>
         </is>
       </c>
-      <c r="AC13" s="3" t="n">
+      <c r="AD13" s="3" t="n">
         <v>2.69</v>
       </c>
-      <c r="AD13" s="3" t="n">
+      <c r="AE13" s="3" t="n">
         <v>0.99</v>
       </c>
-      <c r="AE13" s="6" t="n">
+      <c r="AF13" s="6" t="n">
         <v>51</v>
       </c>
     </row>
@@ -2047,27 +2113,32 @@
       <c r="X14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y14" s="6" t="n">
+      <c r="Y14" s="6" t="inlineStr">
+        <is>
+          <t>0/52</t>
+        </is>
+      </c>
+      <c r="Z14" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="Z14" s="6" t="n">
+      <c r="AA14" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="AA14" s="6" t="n">
+      <c r="AB14" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="AB14" s="2" t="inlineStr">
+      <c r="AC14" s="2" t="inlineStr">
         <is>
           <t>Material de Slime (Defectuoso)×1</t>
         </is>
       </c>
-      <c r="AC14" s="3" t="n">
+      <c r="AD14" s="3" t="n">
         <v>2.82</v>
       </c>
-      <c r="AD14" s="3" t="n">
+      <c r="AE14" s="3" t="n">
         <v>1.02</v>
       </c>
-      <c r="AE14" s="6" t="n">
+      <c r="AF14" s="6" t="n">
         <v>52</v>
       </c>
     </row>
@@ -2150,27 +2221,32 @@
       <c r="X15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y15" s="6" t="n">
+      <c r="Y15" s="6" t="inlineStr">
+        <is>
+          <t>0/52</t>
+        </is>
+      </c>
+      <c r="Z15" s="6" t="n">
         <v>2</v>
-      </c>
-      <c r="Z15" s="6" t="n">
-        <v>3</v>
       </c>
       <c r="AA15" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="AB15" s="2" t="inlineStr">
+      <c r="AB15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC15" s="2" t="inlineStr">
         <is>
           <t>ninguno</t>
         </is>
       </c>
-      <c r="AC15" s="3" t="n">
+      <c r="AD15" s="3" t="n">
         <v>2.43</v>
       </c>
-      <c r="AD15" s="3" t="n">
+      <c r="AE15" s="3" t="n">
         <v>0.98</v>
       </c>
-      <c r="AE15" s="6" t="n">
+      <c r="AF15" s="6" t="n">
         <v>52</v>
       </c>
     </row>
@@ -2253,27 +2329,32 @@
       <c r="X16" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y16" s="6" t="n">
+      <c r="Y16" s="6" t="inlineStr">
+        <is>
+          <t>0/45</t>
+        </is>
+      </c>
+      <c r="Z16" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="Z16" s="6" t="n">
+      <c r="AA16" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AA16" s="6" t="n">
+      <c r="AB16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB16" s="2" t="inlineStr">
+      <c r="AC16" s="2" t="inlineStr">
         <is>
           <t>Material de Slime (Defectuoso)×1 (+1 cristal roto/perdido, no contabilizado)</t>
         </is>
       </c>
-      <c r="AC16" s="3" t="n">
+      <c r="AD16" s="3" t="n">
         <v>2.91</v>
       </c>
-      <c r="AD16" s="3" t="n">
+      <c r="AE16" s="3" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="AE16" s="6" t="n">
+      <c r="AF16" s="6" t="n">
         <v>45</v>
       </c>
     </row>
@@ -2356,27 +2437,32 @@
       <c r="X17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y17" s="6" t="n">
+      <c r="Y17" s="6" t="inlineStr">
+        <is>
+          <t>0/41</t>
+        </is>
+      </c>
+      <c r="Z17" s="6" t="n">
         <v>1</v>
-      </c>
-      <c r="Z17" s="6" t="n">
-        <v>3</v>
       </c>
       <c r="AA17" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="AB17" s="2" t="inlineStr">
+      <c r="AB17" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC17" s="2" t="inlineStr">
         <is>
           <t>ninguno (+1 cristal roto/perdido, no contabilizado)</t>
         </is>
       </c>
-      <c r="AC17" s="3" t="n">
+      <c r="AD17" s="3" t="n">
         <v>2.59</v>
       </c>
-      <c r="AD17" s="3" t="n">
+      <c r="AE17" s="3" t="n">
         <v>1.09</v>
       </c>
-      <c r="AE17" s="6" t="n">
+      <c r="AF17" s="6" t="n">
         <v>41</v>
       </c>
     </row>
@@ -2459,27 +2545,32 @@
       <c r="X18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y18" s="6" t="n">
+      <c r="Y18" s="6" t="inlineStr">
+        <is>
+          <t>0/42</t>
+        </is>
+      </c>
+      <c r="Z18" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Z18" s="6" t="n">
+      <c r="AA18" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AA18" s="6" t="n">
+      <c r="AB18" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="AB18" s="2" t="inlineStr">
+      <c r="AC18" s="2" t="inlineStr">
         <is>
           <t>ninguno</t>
         </is>
       </c>
-      <c r="AC18" s="3" t="n">
+      <c r="AD18" s="3" t="n">
         <v>2.61</v>
       </c>
-      <c r="AD18" s="3" t="n">
+      <c r="AE18" s="3" t="n">
         <v>1.03</v>
       </c>
-      <c r="AE18" s="6" t="n">
+      <c r="AF18" s="6" t="n">
         <v>42</v>
       </c>
     </row>
@@ -2562,41 +2653,840 @@
       <c r="X19" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y19" s="6" t="n">
+      <c r="Y19" s="6" t="inlineStr">
+        <is>
+          <t>0/43</t>
+        </is>
+      </c>
+      <c r="Z19" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="Z19" s="6" t="n">
+      <c r="AA19" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="AA19" s="6" t="n">
+      <c r="AB19" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AB19" s="2" t="inlineStr">
+      <c r="AC19" s="2" t="inlineStr">
         <is>
           <t>Material de Slime (Defectuoso)×1</t>
         </is>
       </c>
-      <c r="AC19" s="3" t="n">
+      <c r="AD19" s="3" t="n">
         <v>2.69</v>
       </c>
-      <c r="AD19" s="3" t="n">
+      <c r="AE19" s="3" t="n">
         <v>1.06</v>
       </c>
-      <c r="AE19" s="6" t="n">
+      <c r="AF19" s="6" t="n">
         <v>43</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña + —</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>6.59</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>513.1</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="6" t="n"/>
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N20" s="6" t="inlineStr">
+        <is>
+          <t>6/7/6/1/0</t>
+        </is>
+      </c>
+      <c r="O20" s="6" t="inlineStr">
+        <is>
+          <t>10/12/9/1/0</t>
+        </is>
+      </c>
+      <c r="P20" s="6" t="inlineStr">
+        <is>
+          <t>16/19/13/3/0</t>
+        </is>
+      </c>
+      <c r="Q20" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="R20" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="S20" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="T20" s="6" t="inlineStr">
+        <is>
+          <t>4.99–6.31 → 5.37–6.55</t>
+        </is>
+      </c>
+      <c r="U20" s="6" t="inlineStr"/>
+      <c r="V20" s="6" t="inlineStr">
+        <is>
+          <t>2.00–2.28</t>
+        </is>
+      </c>
+      <c r="W20" s="6" t="inlineStr">
+        <is>
+          <t>2.52–3.36</t>
+        </is>
+      </c>
+      <c r="X20" s="5" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="Y20" s="6" t="inlineStr">
+        <is>
+          <t>3/57</t>
+        </is>
+      </c>
+      <c r="Z20" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA20" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC20" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AD20" s="3" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="AE20" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AF20" s="6" t="n">
+        <v>57</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>* Mano 2 idéntica a Mano 1: el log de Daga+Daga(dual) no distingue qué mano golpeó en cada línea (mismo arma en ambas manos).</t>
-        </is>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña + Daga (dual)</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>730.4</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Daga</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="J21" s="5" t="n">
+        <v>0.926</v>
+      </c>
+      <c r="K21" s="5" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="M21" s="3" t="n">
+        <v>1.475</v>
+      </c>
+      <c r="N21" s="6" t="inlineStr">
+        <is>
+          <t>5/5/2/1/0</t>
+        </is>
+      </c>
+      <c r="O21" s="6" t="inlineStr">
+        <is>
+          <t>9/10/7/3/0</t>
+        </is>
+      </c>
+      <c r="P21" s="6" t="inlineStr">
+        <is>
+          <t>15/16/12/5/0</t>
+        </is>
+      </c>
+      <c r="Q21" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="R21" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="S21" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="T21" s="6" t="inlineStr">
+        <is>
+          <t>5.06–6.23 → 5.35–6.56</t>
+        </is>
+      </c>
+      <c r="U21" s="6" t="inlineStr">
+        <is>
+          <t>4.09–5.03 → 5.01–5.44</t>
+        </is>
+      </c>
+      <c r="V21" s="6" t="inlineStr">
+        <is>
+          <t>1.75–2.16</t>
+        </is>
+      </c>
+      <c r="W21" s="6" t="inlineStr">
+        <is>
+          <t>2.67–3.40</t>
+        </is>
+      </c>
+      <c r="X21" s="5" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="Y21" s="6" t="inlineStr">
+        <is>
+          <t>4/32</t>
+        </is>
+      </c>
+      <c r="Z21" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA21" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB21" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC21" s="2" t="inlineStr">
+        <is>
+          <t>ninguno (+1 cristal roto/perdido, no contabilizado)</t>
+        </is>
+      </c>
+      <c r="AD21" s="3" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="AE21" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AF21" s="6" t="n">
+        <v>59</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>% Aturdir proc solo cuenta golpes de la mano capaz de aturdir (aturdir base &gt; 0); las demás manos siempre dan 0%.</t>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña + Espada corta (dual)</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>744.7</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>5.21</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>0.857</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Espada corta</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="J22" s="5" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="K22" s="5" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="M22" s="3" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="N22" s="6" t="inlineStr">
+        <is>
+          <t>4/4/4/1/0</t>
+        </is>
+      </c>
+      <c r="O22" s="6" t="inlineStr">
+        <is>
+          <t>8/8/8/3/0</t>
+        </is>
+      </c>
+      <c r="P22" s="6" t="inlineStr">
+        <is>
+          <t>13/13/13/5/0</t>
+        </is>
+      </c>
+      <c r="Q22" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="R22" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="S22" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="T22" s="6" t="inlineStr">
+        <is>
+          <t>5.23–6.15 → 5.41–6.67</t>
+        </is>
+      </c>
+      <c r="U22" s="6" t="inlineStr">
+        <is>
+          <t>5.37–6.15 → 5.59–6.94</t>
+        </is>
+      </c>
+      <c r="V22" s="6" t="inlineStr">
+        <is>
+          <t>1.54–1.87</t>
+        </is>
+      </c>
+      <c r="W22" s="6" t="inlineStr">
+        <is>
+          <t>2.55–3.37</t>
+        </is>
+      </c>
+      <c r="X22" s="5" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="Y22" s="6" t="inlineStr">
+        <is>
+          <t>2/28</t>
+        </is>
+      </c>
+      <c r="Z22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA22" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB22" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC22" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AD22" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AE22" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="AF22" s="6" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña + Maza pequeña (dual)</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>704.9</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña*</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="J23" s="5" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="K23" s="5" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="L23" s="3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M23" s="3" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
+          <t>4/3/5/1/0</t>
+        </is>
+      </c>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>7/7/9/2/0</t>
+        </is>
+      </c>
+      <c r="P23" s="6" t="inlineStr">
+        <is>
+          <t>14/13/13/3/0</t>
+        </is>
+      </c>
+      <c r="Q23" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="R23" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="S23" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="T23" s="6" t="inlineStr">
+        <is>
+          <t>5.10–6.37 → 5.36–6.56</t>
+        </is>
+      </c>
+      <c r="U23" s="6" t="inlineStr"/>
+      <c r="V23" s="6" t="inlineStr">
+        <is>
+          <t>1.56–1.84</t>
+        </is>
+      </c>
+      <c r="W23" s="6" t="inlineStr">
+        <is>
+          <t>2.65–3.37</t>
+        </is>
+      </c>
+      <c r="X23" s="5" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="Y23" s="6" t="inlineStr">
+        <is>
+          <t>6/52</t>
+        </is>
+      </c>
+      <c r="Z23" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC23" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AD23" s="3" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="AE23" s="3" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="AF23" s="6" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña + Escudo pequeño</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>534.9</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="6" t="n"/>
+      <c r="J24" s="6" t="n"/>
+      <c r="K24" s="6" t="n"/>
+      <c r="L24" s="3" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="M24" s="3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="N24" s="6" t="inlineStr">
+        <is>
+          <t>5/6/6/1/0</t>
+        </is>
+      </c>
+      <c r="O24" s="6" t="inlineStr">
+        <is>
+          <t>10/14/12/3/0</t>
+        </is>
+      </c>
+      <c r="P24" s="6" t="inlineStr">
+        <is>
+          <t>14/17/14/4/0</t>
+        </is>
+      </c>
+      <c r="Q24" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="R24" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="S24" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="T24" s="6" t="inlineStr">
+        <is>
+          <t>5.03–6.29 → 5.32–6.63</t>
+        </is>
+      </c>
+      <c r="U24" s="6" t="inlineStr"/>
+      <c r="V24" s="6" t="inlineStr">
+        <is>
+          <t>1.15–1.48</t>
+        </is>
+      </c>
+      <c r="W24" s="6" t="inlineStr">
+        <is>
+          <t>2.57–3.38</t>
+        </is>
+      </c>
+      <c r="X24" s="5" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="Y24" s="6" t="inlineStr">
+        <is>
+          <t>4/50</t>
+        </is>
+      </c>
+      <c r="Z24" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA24" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB24" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC24" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AD24" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="AE24" s="3" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AF24" s="6" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña + Escudo normal</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>493.3</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="6" t="n"/>
+      <c r="J25" s="6" t="n"/>
+      <c r="K25" s="6" t="n"/>
+      <c r="L25" s="3" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="M25" s="3" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="N25" s="6" t="inlineStr">
+        <is>
+          <t>5/9/6/1/0</t>
+        </is>
+      </c>
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>11/20/11/2/0</t>
+        </is>
+      </c>
+      <c r="P25" s="6" t="inlineStr">
+        <is>
+          <t>14/25/13/3/0</t>
+        </is>
+      </c>
+      <c r="Q25" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="R25" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="S25" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="T25" s="6" t="inlineStr">
+        <is>
+          <t>5.21–6.23 → 5.51–6.77</t>
+        </is>
+      </c>
+      <c r="U25" s="6" t="inlineStr"/>
+      <c r="V25" s="6" t="inlineStr">
+        <is>
+          <t>0.91–1.17</t>
+        </is>
+      </c>
+      <c r="W25" s="6" t="inlineStr">
+        <is>
+          <t>2.51–3.34</t>
+        </is>
+      </c>
+      <c r="X25" s="5" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="Y25" s="6" t="inlineStr">
+        <is>
+          <t>7/50</t>
+        </is>
+      </c>
+      <c r="Z25" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA25" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC25" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AD25" s="3" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="AE25" s="3" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="AF25" s="6" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña + Escudo grande</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>397.2</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Maza pequeña</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>0.842</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="6" t="n"/>
+      <c r="J26" s="6" t="n"/>
+      <c r="K26" s="6" t="n"/>
+      <c r="L26" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M26" s="3" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="N26" s="6" t="inlineStr">
+        <is>
+          <t>5/11/3/2/0</t>
+        </is>
+      </c>
+      <c r="O26" s="6" t="inlineStr">
+        <is>
+          <t>10/19/7/2/0</t>
+        </is>
+      </c>
+      <c r="P26" s="6" t="inlineStr">
+        <is>
+          <t>15/28/11/4/0</t>
+        </is>
+      </c>
+      <c r="Q26" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="R26" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="S26" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="T26" s="6" t="inlineStr">
+        <is>
+          <t>5.08–6.35 → 5.32–6.68</t>
+        </is>
+      </c>
+      <c r="U26" s="6" t="inlineStr"/>
+      <c r="V26" s="6" t="inlineStr">
+        <is>
+          <t>0.64–0.74</t>
+        </is>
+      </c>
+      <c r="W26" s="6" t="inlineStr">
+        <is>
+          <t>2.68–3.42</t>
+        </is>
+      </c>
+      <c r="X26" s="5" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="Y26" s="6" t="inlineStr">
+        <is>
+          <t>7/57</t>
+        </is>
+      </c>
+      <c r="Z26" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB26" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC26" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AD26" s="3" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="AE26" s="3" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="AF26" s="6" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>* Mano 2 idéntica a Mano 1: el log de armas iguales en ambas manos no distingue qué mano golpeó en cada línea.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>% Aturdir proc / Aturdir proc (n/n) solo cuentan golpes de la mano capaz de aturdir (aturdir base &gt; 0); las demás manos siempre dan 0%.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Balance Mandobles/Hacha grande (dos manos) + Excel pruebas completo
Las dos manos pesadas igualaban o superaban el DPS del mejor dual-wield
ligero mientras conservaban un bloqueo mucho más alto, sin ningún
trade-off real. Se les baja MV y bloqueo (Mandobles algo menos que
Hacha, para no invertir su orden relativo), dejando su DPS por debajo
del mejor dual ligero. Martillo grande no se toca: ya paga su alto
bloqueo/aturdir con menos DPS.

Incluye el Excel actualizado (28 filas: Daga, Espada corta, Espada
larga, Maza pequeña completas + Mandobles y Hacha grande re-probadas
con el nuevo balance).
</commit_message>
<xml_diff>
--- a/pruebas_combos_slime.xlsx
+++ b/pruebas_combos_slime.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF29"/>
+  <dimension ref="A1:AF32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3476,15 +3476,339 @@
         <v>57</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Mandobles + —</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>12.69</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>682</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Mandobles</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>10.18</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>0.897</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="6" t="n"/>
+      <c r="J27" s="6" t="n"/>
+      <c r="K27" s="6" t="n"/>
+      <c r="L27" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M27" s="3" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="N27" s="6" t="inlineStr">
+        <is>
+          <t>3/3/2/1/0</t>
+        </is>
+      </c>
+      <c r="O27" s="6" t="inlineStr">
+        <is>
+          <t>10/11/9/3/0</t>
+        </is>
+      </c>
+      <c r="P27" s="6" t="inlineStr">
+        <is>
+          <t>13/14/11/4/0</t>
+        </is>
+      </c>
+      <c r="Q27" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="R27" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="S27" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="T27" s="6" t="inlineStr">
+        <is>
+          <t>9.81–12.36 → 10.47–12.56</t>
+        </is>
+      </c>
+      <c r="U27" s="6" t="inlineStr"/>
+      <c r="V27" s="6" t="inlineStr">
+        <is>
+          <t>1.34–1.61</t>
+        </is>
+      </c>
+      <c r="W27" s="6" t="inlineStr">
+        <is>
+          <t>2.64–3.39</t>
+        </is>
+      </c>
+      <c r="X27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y27" s="6" t="inlineStr">
+        <is>
+          <t>0/29</t>
+        </is>
+      </c>
+      <c r="Z27" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB27" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC27" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AD27" s="3" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="AE27" s="3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="AF27" s="6" t="n">
+        <v>29</v>
+      </c>
+    </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>* Mano 2 idéntica a Mano 1: el log de armas iguales en ambas manos no distingue qué mano golpeó en cada línea.</t>
-        </is>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Hacha grande + —</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>13.04</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>757</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Hacha grande</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>12.21</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="6" t="n"/>
+      <c r="J28" s="6" t="n"/>
+      <c r="K28" s="6" t="n"/>
+      <c r="L28" s="3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="M28" s="3" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="N28" s="6" t="inlineStr">
+        <is>
+          <t>3/5/4/1/0</t>
+        </is>
+      </c>
+      <c r="O28" s="6" t="inlineStr">
+        <is>
+          <t>6/9/6/3/0</t>
+        </is>
+      </c>
+      <c r="P28" s="6" t="inlineStr">
+        <is>
+          <t>10/14/10/6/0</t>
+        </is>
+      </c>
+      <c r="Q28" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="R28" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="S28" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="T28" s="6" t="inlineStr">
+        <is>
+          <t>10.38–11.97 → 10.66–13.35</t>
+        </is>
+      </c>
+      <c r="U28" s="6" t="inlineStr"/>
+      <c r="V28" s="6" t="inlineStr">
+        <is>
+          <t>1.44–1.73</t>
+        </is>
+      </c>
+      <c r="W28" s="6" t="inlineStr">
+        <is>
+          <t>2.54–3.33</t>
+        </is>
+      </c>
+      <c r="X28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="6" t="inlineStr">
+        <is>
+          <t>0/25</t>
+        </is>
+      </c>
+      <c r="Z28" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA28" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC28" s="2" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+      <c r="AD28" s="3" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="AE28" s="3" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="AF28" s="6" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Martillo grande + —</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>13.99</v>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>566.7</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Martillo grande</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>0.828</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="6" t="n"/>
+      <c r="J29" s="6" t="n"/>
+      <c r="K29" s="6" t="n"/>
+      <c r="L29" s="3" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="M29" s="3" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="N29" s="6" t="inlineStr">
+        <is>
+          <t>4/6/2/3/0</t>
+        </is>
+      </c>
+      <c r="O29" s="6" t="inlineStr">
+        <is>
+          <t>10/14/7/4/0</t>
+        </is>
+      </c>
+      <c r="P29" s="6" t="inlineStr">
+        <is>
+          <t>15/20/11/7/0</t>
+        </is>
+      </c>
+      <c r="Q29" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="R29" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="S29" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="T29" s="6" t="inlineStr">
+        <is>
+          <t>10.84–13.31 → 11.42–14.17</t>
+        </is>
+      </c>
+      <c r="U29" s="6" t="inlineStr"/>
+      <c r="V29" s="6" t="inlineStr">
+        <is>
+          <t>1.28–1.61</t>
+        </is>
+      </c>
+      <c r="W29" s="6" t="inlineStr">
+        <is>
+          <t>2.58–3.46</t>
+        </is>
+      </c>
+      <c r="X29" s="5" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="Y29" s="6" t="inlineStr">
+        <is>
+          <t>7/29</t>
+        </is>
+      </c>
+      <c r="Z29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB29" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC29" s="2" t="inlineStr">
+        <is>
+          <t>ninguno (+1 cristal roto/perdido, no contabilizado)</t>
+        </is>
+      </c>
+      <c r="AD29" s="3" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="AE29" s="3" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="AF29" s="6" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>* Mano 2 idéntica a Mano 1: el log de armas iguales en ambas manos no distingue qué mano golpeó en cada línea.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>% Aturdir proc / Aturdir proc (n/n) solo cuentan golpes de la mano capaz de aturdir (aturdir base &gt; 0); las demás manos siempre dan 0%.</t>
         </is>

</xml_diff>